<commit_message>
Added Loggers, ExtentReports, Screenshot using listners
</commit_message>
<xml_diff>
--- a/testData/LoginData.xlsx
+++ b/testData/LoginData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\AutomationFramework\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34B6566F-1106-497A-901E-E19779D7AD52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40C2802F-AA29-4AB3-B66A-15676BD66301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{DC25A50C-6C16-40B4-B2BC-F74BC89B73EC}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>email</t>
   </si>
@@ -45,10 +45,7 @@
     <t>fipad42714@pazard.com</t>
   </si>
   <si>
-    <t>Admin@1234</t>
-  </si>
-  <si>
-    <t>Ajdhhj@12393</t>
+    <t>Admin@123439</t>
   </si>
 </sst>
 </file>
@@ -418,7 +415,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04BCCC4D-F5D0-4DBA-8FD1-FEC16340E2B4}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22.07421875" bestFit="1" customWidth="1"/>
@@ -438,20 +435,12 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
         <v>3</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" xr:uid="{6A89288C-9314-4E15-97CB-784721AE610E}"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{06180389-994F-43B0-9C50-9437B54192D4}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Cloud test, parallel execution using testng.xml, parameterize testng.xml
</commit_message>
<xml_diff>
--- a/testData/LoginData.xlsx
+++ b/testData/LoginData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Eclipse\AutomationFramework\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40C2802F-AA29-4AB3-B66A-15676BD66301}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55E21B0A-8287-4BB6-9E19-D1590E1C7B24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{DC25A50C-6C16-40B4-B2BC-F74BC89B73EC}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="5">
   <si>
     <t>email</t>
   </si>
@@ -46,6 +46,9 @@
   </si>
   <si>
     <t>Admin@123439</t>
+  </si>
+  <si>
+    <t>Admin@1234</t>
   </si>
 </sst>
 </file>
@@ -415,7 +418,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04BCCC4D-F5D0-4DBA-8FD1-FEC16340E2B4}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="22.07421875" bestFit="1" customWidth="1"/>
@@ -438,9 +441,18 @@
         <v>3</v>
       </c>
     </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{06180389-994F-43B0-9C50-9437B54192D4}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{21466710-0D0F-4B6C-8A15-BDDBC3CE71F6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>